<commit_message>
Replace PersonalInformation with Profile entity
Refactored the domain to use a new Profile entity for both Customer and Employee, replacing all references to PersonalInformation. Updated navigation properties, foreign keys, repositories, services, and DTOs accordingly. Removed PersonalInformation-related files and introduced Profile repository, configuration, and seeder. Updated database context, migrations, dependency injection, and Excel seeding logic to support the new Profile model.
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30219"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30306"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="69" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17ED05FC-D835-4661-9EAC-ED6A10D4CBC5}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C0F6651-47CF-47C7-9E80-3587A84FBE1F}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="8" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
     <sheet name="Areas" sheetId="2" r:id="rId2"/>
-    <sheet name="PersonalInformations" sheetId="3" r:id="rId3"/>
+    <sheet name="Profile" sheetId="3" r:id="rId3"/>
     <sheet name="Images" sheetId="4" r:id="rId4"/>
     <sheet name="Roles" sheetId="5" r:id="rId5"/>
     <sheet name="Products" sheetId="6" r:id="rId6"/>
@@ -1015,7 +1015,7 @@
     <t>UserId</t>
   </si>
   <si>
-    <t>PIId</t>
+    <t>ProfileId</t>
   </si>
   <si>
     <t>770e8400-e29b-41d4-a716-446655440001</t>

</xml_diff>